<commit_message>
mais um dicionario novo
</commit_message>
<xml_diff>
--- a/Estudando/excel/dicionario_de_dados.xlsx
+++ b/Estudando/excel/dicionario_de_dados.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L39"/>
+  <dimension ref="A1:K39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -439,40 +439,35 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Tamanho</t>
+          <t>Nulo</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Nulo</t>
+          <t>PK</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>PK</t>
+          <t>FK</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>FK</t>
+          <t>Unique</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>Unique</t>
+          <t>Identity</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
-        <is>
-          <t>Default</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
         <is>
           <t>Restrições</t>
         </is>
@@ -481,404 +476,333 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>USUARIO</t>
+          <t>ENDERECO</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>nome</t>
+          <t>rua</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>varchar</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>255</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>NAO</t>
-        </is>
-      </c>
+          <t>NAO</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>USUARIO</t>
+          <t>ENDERECO</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>email_usuario</t>
+          <t>pais</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>255</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>NAO</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
+          <t>NAO</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
+      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>PRIMARY KEY, UNIQUE</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>USUARIO</t>
+          <t>ENDERECO</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>senha</t>
+          <t>bairro</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>password_hash</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>255</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>NAO</t>
-        </is>
-      </c>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>USUARIO</t>
+          <t>ENDERECO</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>login</t>
+          <t>cep</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>NAO</t>
-        </is>
-      </c>
+          <t>NAO</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>USUARIO</t>
+          <t>ENDERECO</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>matricula</t>
+          <t>numero</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
+          <t>NAO</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ORIENTADOR</t>
+          <t>ENDERECO</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>email_usuario</t>
+          <t>cidade</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>255</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>NAO</t>
-        </is>
-      </c>
+          <t>NAO</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>USUARIO(email_usuario)</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>FOREIGN KEY, UNIQUE</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>FASE</t>
+          <t>ENDERECO</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>pds</t>
+          <t>estado</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>NAO</t>
-        </is>
-      </c>
+          <t>NAO</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>STATUS</t>
+          <t>ENDERECO</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>momento</t>
+          <t>tipo_casa</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>NAO</t>
-        </is>
-      </c>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>PROJETO</t>
+          <t>ENDERECO</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>avaliacao</t>
+          <t>id_endereco</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>NAO</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>NAO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>PRIMARY KEY</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>PROJETO</t>
+          <t>CLIENTE</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>descricao</t>
+          <t>tipo_pessoa</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>max</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>NAO</t>
-        </is>
-      </c>
+          <t>NAO</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>PROJETO</t>
+          <t>CLIENTE</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>titulo_projeto</t>
+          <t>cpf</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>varchar</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>NAO</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>NAO</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
           <t>SIM</t>
         </is>
       </c>
+      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>PRIMARY KEY</t>
         </is>
@@ -887,1092 +811,869 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>PROJETO</t>
+          <t>CLIENTE</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>data_criacao</t>
+          <t>telefone</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>datetime</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>NAO</t>
-        </is>
-      </c>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>NAO</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>PROJETO</t>
+          <t>CLIENTE</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>data_finalizacao</t>
+          <t>email</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>datetime</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>NAO</t>
-        </is>
-      </c>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>NAO</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>PROJETO</t>
+          <t>CLIENTE</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>data_publicacao</t>
+          <t>id_endereco</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>datetime</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>NAO</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr"/>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>NAO</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>ENDERECO(id_endereco)</t>
+        </is>
+      </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>FOREIGN KEY</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>PROJETO</t>
+          <t>PRODUTO</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>resumo</t>
+          <t>nome_produto</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>max</t>
+          <t>NAO</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>NAO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>PRIMARY KEY</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>PROJETO</t>
+          <t>PRODUTO</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>imagem</t>
+          <t>preco_produto</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>NAO</t>
-        </is>
-      </c>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>NAO</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>PROJETO</t>
+          <t>PRODUTO</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>repositorio</t>
+          <t>observacoes</t>
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>NAO</t>
-        </is>
-      </c>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ORIENTANDO</t>
+          <t>PRODUTO</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>matrícula_orientando</t>
+          <t>quantidade</t>
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>NAO</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
+          <t>NAO</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>PRIMARY KEY</t>
-        </is>
-      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ORIENTANDO</t>
+          <t>PRODUTO</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>subtotal_produto</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>255</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>NAO</t>
-        </is>
-      </c>
+          <t>NAO</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>USUARIO(email_usuario)</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>FOREIGN KEY, UNIQUE</t>
-        </is>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>PLATAFORMA</t>
+          <t>FRETE</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>tipo</t>
+          <t>preco_frete</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>NAO</t>
-        </is>
-      </c>
+          <t>NAO</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>TECNOLOGIA</t>
+          <t>FRETE</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>nome</t>
+          <t>dh_entrega</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
-          <t>varchar</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>255</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>NAO</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
+          <t>NAO</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>PRIMARY KEY</t>
-        </is>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>TECNOLOGIA</t>
+          <t>FRETE</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>icone</t>
+          <t>empresa_envio</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>NAO</t>
-        </is>
-      </c>
+          <t>NAO</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>AVALIAR</t>
+          <t>FRETE</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>nota</t>
+          <t>id_frete</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>NAO</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>NAO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>PRIMARY KEY</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>AVALIAR</t>
+          <t>PAGAMENTO</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>comentario</t>
+          <t>tipos_pagamento</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>max</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>NAO</t>
-        </is>
-      </c>
+          <t>NAO</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>AVALIAR</t>
+          <t>PAGAMENTO</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>titulo_projeto</t>
+          <t>numero_cartao</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
-          <t>varchar</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>255</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>NAO</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>PROJETO(titulo_projeto)</t>
-        </is>
-      </c>
+          <t>NAO</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>PRIMARY KEY, FOREIGN KEY</t>
-        </is>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>AVALIAR</t>
+          <t>PAGAMENTO</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>email_usuario</t>
+          <t>nome_titular</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>255</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>NAO</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>USUARIO(email_usuario)</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
+          <t>NAO</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>PRIMARY KEY, FOREIGN KEY, UNIQUE</t>
-        </is>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>PARTICIPA</t>
+          <t>PAGAMENTO</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>situacao</t>
+          <t>vencimento</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>NAO</t>
-        </is>
-      </c>
+          <t>NAO</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>PARTICIPA</t>
+          <t>PAGAMENTO</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>matrícula_orientando</t>
+          <t>codigo_seguranca</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>NAO</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>ORIENTANDO(matrícula_orientando)</t>
-        </is>
-      </c>
+          <t>NAO</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr">
-        <is>
-          <t>PRIMARY KEY, FOREIGN KEY</t>
-        </is>
-      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>PARTICIPA</t>
+          <t>PAGAMENTO</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>titulo_projeto</t>
+          <t>id_pagamento</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
-          <t>varchar</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>NAO</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>NAO</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
           <t>SIM</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>PROJETO(titulo_projeto)</t>
-        </is>
-      </c>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr">
-        <is>
-          <t>PRIMARY KEY, FOREIGN KEY</t>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>PRIMARY KEY</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>FAVORITAR</t>
+          <t>CARRINHO</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>titulo_projeto</t>
+          <t>cupom</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr">
         <is>
-          <t>varchar</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>255</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>NAO</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>PROJETO(titulo_projeto)</t>
-        </is>
-      </c>
+          <t>NAO</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr">
-        <is>
-          <t>PRIMARY KEY, FOREIGN KEY</t>
-        </is>
-      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>FAVORITAR</t>
+          <t>CARRINHO</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>email_usuario</t>
+          <t>subtotal_carrinho</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>255</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>NAO</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>USUARIO(email_usuario)</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
+          <t>NAO</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr">
-        <is>
-          <t>PRIMARY KEY, FOREIGN KEY, UNIQUE</t>
-        </is>
-      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CATEGORIA</t>
+          <t>CARRINHO</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>id_principal</t>
+          <t>total_carrinho</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>NAO</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>PROJETO(titulo_projeto)</t>
-        </is>
-      </c>
+          <t>NAO</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
+      <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr">
-        <is>
-          <t>PRIMARY KEY, FOREIGN KEY</t>
-        </is>
-      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CATEGORIA</t>
+          <t>CARRINHO</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>id_subcategoria</t>
+          <t>id_carrinho</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>NAO</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>NAO</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
           <t>SIM</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>PROJETO(titulo_projeto)</t>
-        </is>
-      </c>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr">
-        <is>
-          <t>PRIMARY KEY, FOREIGN KEY</t>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>PRIMARY KEY</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ASSOCIADO</t>
+          <t>CARRINHO</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>titulo_projeto</t>
+          <t>cpf</t>
         </is>
       </c>
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
-          <t>varchar</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>255</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>NAO</t>
-        </is>
-      </c>
+          <t>NAO</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>PROJETO(titulo_projeto)</t>
-        </is>
-      </c>
+          <t>CLIENTE(cpf)</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr">
-        <is>
-          <t>PRIMARY KEY, FOREIGN KEY</t>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>FOREIGN KEY</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>POSSUI</t>
+          <t>CARRINHO</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>nome_tecnologia</t>
+          <t>id_frete</t>
         </is>
       </c>
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr">
         <is>
-          <t>varchar</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>255</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>NAO</t>
-        </is>
-      </c>
+          <t>NAO</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
         <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>TECNOLOGIA(nome)</t>
-        </is>
-      </c>
+          <t>FRETE(id_frete)</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr">
-        <is>
-          <t>PRIMARY KEY, FOREIGN KEY</t>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>FOREIGN KEY</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>POSSUI</t>
+          <t>CARRINHO</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>titulo_projeto</t>
+          <t>id_pagamento</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
-          <t>varchar</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>255</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>NAO</t>
-        </is>
-      </c>
+          <t>NAO</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>PROJETO(titulo_projeto)</t>
-        </is>
-      </c>
+          <t>PAGAMENTO(id_pagamento)</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr">
-        <is>
-          <t>PRIMARY KEY, FOREIGN KEY</t>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>FOREIGN KEY</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>PROJETO_CONTATO</t>
+          <t>TEM</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>contato</t>
+          <t>id_carrinho</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>NAO</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>NAO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>CARRINHO(id_carrinho)</t>
         </is>
       </c>
       <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr">
-        <is>
-          <t>PRIMARY KEY</t>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>PRIMARY KEY, FOREIGN KEY</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>PROJETO_CONTATO</t>
+          <t>TEM</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>titulo</t>
+          <t>nome_produto</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
-          <t>varchar</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>NAO</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>NAO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>PROJETO(titulo_projeto)</t>
-        </is>
-      </c>
+          <t>PRODUTO(nome_produto)</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr">
+      <c r="K39" t="inlineStr">
         <is>
           <t>PRIMARY KEY, FOREIGN KEY</t>
         </is>

</xml_diff>